<commit_message>
data: stage coverage refresh 3/6
</commit_message>
<xml_diff>
--- a/diseases/d014/2010-2014.xlsx
+++ b/diseases/d014/2010-2014.xlsx
@@ -7049,28 +7049,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO43" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP43" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR43" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS43" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ43" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS43" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU43" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV43" t="inlineStr">
@@ -7197,28 +7211,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO44" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP44" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR44" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS44" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ44" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS44" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU44" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV44" t="inlineStr">
@@ -7345,28 +7373,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO45" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP45" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR45" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS45" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ45" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS45" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU45" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV45" t="inlineStr">
@@ -7493,28 +7535,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO46" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP46" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR46" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS46" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ46" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS46" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU46" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV46" t="inlineStr">
@@ -7641,28 +7697,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO47" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP47" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR47" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS47" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ47" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS47" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU47" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV47" t="inlineStr">
@@ -7942,28 +8012,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO49" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP49" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR49" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS49" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ49" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS49" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU49" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV49" t="inlineStr">
@@ -8090,28 +8174,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO50" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP50" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR50" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS50" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ50" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS50" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU50" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV50" t="inlineStr">
@@ -8238,28 +8336,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO51" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP51" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR51" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS51" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ51" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS51" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU51" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV51" t="inlineStr">
@@ -8386,28 +8498,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO52" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP52" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR52" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS52" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ52" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS52" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU52" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV52" t="inlineStr">
@@ -8687,28 +8813,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO54" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP54" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR54" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS54" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ54" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS54" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU54" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV54" t="inlineStr">
@@ -8835,28 +8975,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO55" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP55" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR55" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS55" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ55" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS55" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU55" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV55" t="inlineStr">
@@ -8983,28 +9137,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO56" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP56" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR56" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS56" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ56" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS56" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU56" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV56" t="inlineStr">
@@ -9131,28 +9299,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO57" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP57" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR57" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS57" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ57" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS57" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU57" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV57" t="inlineStr">
@@ -9432,28 +9614,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO59" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP59" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR59" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS59" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ59" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS59" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU59" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV59" t="inlineStr">
@@ -9580,28 +9776,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO60" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP60" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR60" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS60" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ60" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS60" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU60" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV60" t="inlineStr">
@@ -9728,28 +9938,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO61" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP61" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR61" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS61" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ61" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS61" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU61" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV61" t="inlineStr">
@@ -9876,28 +10100,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO62" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP62" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR62" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS62" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ62" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS62" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU62" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV62" t="inlineStr">
@@ -10024,28 +10262,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO63" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP63" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR63" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS63" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ63" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS63" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU63" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV63" t="inlineStr">
@@ -10325,28 +10577,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO65" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP65" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR65" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS65" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ65" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS65" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU65" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV65" t="inlineStr">
@@ -10473,28 +10739,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO66" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP66" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR66" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS66" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ66" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS66" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU66" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV66" t="inlineStr">
@@ -10621,28 +10901,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO67" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP67" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR67" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS67" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ67" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS67" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU67" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV67" t="inlineStr">
@@ -10769,28 +11063,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO68" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP68" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR68" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS68" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ68" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS68" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU68" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV68" t="inlineStr">
@@ -11070,28 +11378,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO70" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP70" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR70" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS70" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ70" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS70" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU70" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV70" t="inlineStr">
@@ -11218,28 +11540,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO71" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP71" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR71" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS71" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ71" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS71" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU71" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV71" t="inlineStr">
@@ -11366,28 +11702,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO72" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP72" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR72" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS72" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ72" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS72" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU72" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV72" t="inlineStr">
@@ -11514,28 +11864,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO73" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP73" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR73" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS73" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ73" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS73" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU73" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV73" t="inlineStr">
@@ -11815,28 +12179,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO75" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP75" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR75" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS75" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ75" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS75" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU75" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV75" t="inlineStr">
@@ -11963,28 +12341,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO76" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP76" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR76" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS76" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ76" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS76" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU76" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV76" t="inlineStr">
@@ -12111,28 +12503,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO77" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP77" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR77" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS77" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ77" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS77" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU77" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV77" t="inlineStr">
@@ -12259,28 +12665,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO78" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP78" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR78" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS78" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ78" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS78" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU78" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV78" t="inlineStr">
@@ -12407,28 +12827,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO79" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP79" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR79" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS79" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ79" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS79" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU79" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV79" t="inlineStr">
@@ -12708,28 +13142,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO81" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP81" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR81" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS81" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ81" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS81" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU81" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV81" t="inlineStr">
@@ -12856,28 +13304,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO82" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP82" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR82" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS82" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ82" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS82" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU82" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV82" t="inlineStr">
@@ -13004,28 +13466,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO83" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP83" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR83" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS83" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ83" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS83" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU83" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV83" t="inlineStr">
@@ -13152,28 +13628,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO84" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP84" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR84" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS84" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ84" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS84" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU84" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV84" t="inlineStr">
@@ -13453,28 +13943,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA86" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO86" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP86" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR86" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS86" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ86" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS86" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU86" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV86" t="inlineStr">
@@ -13601,28 +14105,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO87" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP87" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR87" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS87" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ87" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS87" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU87" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV87" t="inlineStr">
@@ -13749,28 +14267,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA88" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO88" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP88" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR88" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS88" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ88" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS88" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU88" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV88" t="inlineStr">
@@ -13897,28 +14429,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA89" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO89" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP89" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR89" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS89" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ89" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS89" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU89" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV89" t="inlineStr">
@@ -14045,28 +14591,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO90" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP90" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR90" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS90" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ90" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS90" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU90" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV90" t="inlineStr">
@@ -14346,28 +14906,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA92" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO92" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP92" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR92" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS92" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ92" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS92" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU92" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV92" t="inlineStr">
@@ -14494,28 +15068,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA93" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO93" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP93" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR93" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS93" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ93" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS93" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU93" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV93" t="inlineStr">
@@ -14642,28 +15230,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO94" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP94" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR94" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS94" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ94" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS94" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU94" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV94" t="inlineStr">
@@ -14790,28 +15392,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO95" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP95" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR95" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS95" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ95" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS95" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU95" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV95" t="inlineStr">
@@ -15091,28 +15707,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO97" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP97" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR97" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS97" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ97" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS97" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU97" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV97" t="inlineStr">
@@ -15239,28 +15869,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO98" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP98" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR98" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS98" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ98" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS98" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU98" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV98" t="inlineStr">
@@ -15387,28 +16031,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO99" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP99" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR99" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS99" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ99" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS99" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU99" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV99" t="inlineStr">
@@ -15535,28 +16193,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA100" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO100" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP100" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR100" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS100" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ100" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS100" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU100" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV100" t="inlineStr">
@@ -15836,28 +16508,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA102" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO102" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP102" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR102" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS102" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ102" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS102" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT102" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU102" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV102" t="inlineStr">
@@ -15984,28 +16670,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO103" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP103" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR103" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS103" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ103" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS103" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU103" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV103" t="inlineStr">
@@ -16132,28 +16832,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO104" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP104" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR104" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS104" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ104" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS104" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU104" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV104" t="inlineStr">
@@ -16280,28 +16994,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA105" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO105" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP105" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR105" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS105" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ105" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS105" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU105" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV105" t="inlineStr">
@@ -16581,28 +17309,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA107" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO107" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP107" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR107" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS107" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ107" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS107" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU107" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV107" t="inlineStr">
@@ -16729,28 +17471,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA108" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO108" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP108" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR108" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS108" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ108" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS108" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU108" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV108" t="inlineStr">
@@ -16877,28 +17633,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA109" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO109" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP109" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR109" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS109" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ109" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS109" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU109" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV109" t="inlineStr">
@@ -17025,28 +17795,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA110" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO110" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP110" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR110" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS110" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ110" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS110" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT110" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU110" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV110" t="inlineStr">
@@ -17173,28 +17957,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA111" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO111" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP111" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR111" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS111" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ111" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS111" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU111" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV111" t="inlineStr">
@@ -17474,28 +18272,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA113" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO113" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP113" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR113" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS113" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ113" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS113" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU113" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV113" t="inlineStr">
@@ -17622,28 +18434,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA114" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO114" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP114" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR114" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS114" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ114" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS114" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU114" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV114" t="inlineStr">
@@ -17770,28 +18596,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA115" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO115" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP115" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR115" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS115" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ115" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS115" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT115" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU115" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV115" t="inlineStr">
@@ -17918,28 +18758,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA116" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO116" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP116" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR116" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS116" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ116" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS116" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT116" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU116" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV116" t="inlineStr">
@@ -18219,28 +19073,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA118" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO118" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP118" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR118" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS118" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ118" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS118" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU118" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV118" t="inlineStr">
@@ -18367,28 +19235,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA119" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO119" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP119" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR119" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS119" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ119" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS119" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU119" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV119" t="inlineStr">
@@ -18515,28 +19397,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA120" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO120" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP120" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR120" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS120" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ120" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS120" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT120" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU120" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV120" t="inlineStr">
@@ -18663,28 +19559,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA121" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO121" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP121" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR121" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS121" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ121" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS121" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT121" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU121" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV121" t="inlineStr">
@@ -18964,28 +19874,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA123" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO123" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP123" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR123" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS123" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ123" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS123" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU123" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV123" t="inlineStr">
@@ -19112,28 +20036,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA124" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO124" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP124" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR124" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS124" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ124" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS124" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU124" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV124" t="inlineStr">
@@ -19260,28 +20198,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA125" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO125" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP125" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR125" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS125" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ125" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS125" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU125" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV125" t="inlineStr">
@@ -19408,28 +20360,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA126" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO126" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP126" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR126" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS126" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ126" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS126" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU126" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV126" t="inlineStr">
@@ -19556,28 +20522,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA127" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO127" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP127" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR127" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS127" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ127" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS127" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU127" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV127" t="inlineStr">
@@ -19857,28 +20837,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO129" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP129" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR129" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS129" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ129" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS129" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU129" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV129" t="inlineStr">
@@ -20005,28 +20999,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA130" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO130" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP130" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR130" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS130" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ130" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS130" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU130" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV130" t="inlineStr">
@@ -20153,28 +21161,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA131" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO131" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP131" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR131" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS131" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ131" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS131" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU131" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV131" t="inlineStr">
@@ -20301,28 +21323,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA132" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO132" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP132" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR132" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS132" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ132" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS132" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU132" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV132" t="inlineStr">
@@ -20602,28 +21638,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U134" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA134" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO134" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP134" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR134" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS134" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ134" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS134" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT134" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU134" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV134" t="inlineStr">
@@ -20750,28 +21800,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA135" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO135" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP135" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR135" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS135" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ135" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS135" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT135" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU135" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV135" t="inlineStr">
@@ -20898,28 +21962,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA136" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO136" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP136" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR136" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS136" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ136" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS136" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU136" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV136" t="inlineStr">
@@ -21046,28 +22124,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA137" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO137" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP137" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR137" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS137" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ137" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS137" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU137" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV137" t="inlineStr">
@@ -21194,28 +22286,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA138" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO138" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP138" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR138" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS138" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ138" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS138" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU138" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV138" t="inlineStr">
@@ -21495,28 +22601,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA140" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO140" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP140" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR140" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS140" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ140" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS140" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT140" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU140" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV140" t="inlineStr">
@@ -21643,28 +22763,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA141" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO141" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP141" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR141" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS141" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ141" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS141" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU141" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV141" t="inlineStr">
@@ -21791,28 +22925,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA142" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO142" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP142" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR142" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS142" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ142" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS142" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT142" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU142" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV142" t="inlineStr">
@@ -21939,28 +23087,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA143" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO143" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP143" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR143" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS143" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ143" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS143" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU143" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV143" t="inlineStr">
@@ -22240,28 +23402,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA145" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO145" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP145" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR145" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS145" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ145" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS145" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU145" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV145" t="inlineStr">
@@ -22388,28 +23564,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA146" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO146" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP146" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR146" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS146" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ146" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS146" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU146" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV146" t="inlineStr">
@@ -22536,28 +23726,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA147" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO147" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP147" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR147" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS147" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ147" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS147" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU147" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV147" t="inlineStr">
@@ -22684,28 +23888,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
+      <c r="AA148" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO148" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP148" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR148" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS148" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ148" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS148" t="inlineStr">
+        <is>
+          <t>HOLD_JP_e82ee0abd1605c338e084bcf6bf9</t>
+        </is>
+      </c>
       <c r="AT148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU148" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV148" t="inlineStr">

</xml_diff>